<commit_message>
More multi-step strategies experiments
</commit_message>
<xml_diff>
--- a/Res_ConvLSTM/DroughtDataset_model_testing_1749213320_h_1.xlsx
+++ b/Res_ConvLSTM/DroughtDataset_model_testing_1749213320_h_1.xlsx
@@ -652,13 +652,13 @@
     </row>
     <row r="2">
       <c r="A2" t="n">
-        <v>0.0005812589710480458</v>
+        <v>0.008588349805330931</v>
       </c>
       <c r="B2" t="n">
-        <v>0.008529498275473037</v>
+        <v>0.008460022863093525</v>
       </c>
       <c r="C2" t="n">
-        <v>6396483</v>
+        <v>6196071</v>
       </c>
       <c r="D2" t="n">
         <v>0</v>
@@ -679,49 +679,49 @@
         <v>0</v>
       </c>
       <c r="J2" t="n">
-        <v>6396483</v>
+        <v>6196071</v>
       </c>
       <c r="K2" t="n">
-        <v>5013592</v>
+        <v>4690075</v>
       </c>
       <c r="L2" t="n">
-        <v>3362087</v>
+        <v>2916785</v>
       </c>
       <c r="M2" t="n">
-        <v>933271</v>
+        <v>789705</v>
       </c>
       <c r="N2" t="n">
-        <v>76946</v>
+        <v>52153</v>
       </c>
       <c r="O2" t="n">
-        <v>512734</v>
+        <v>458320</v>
       </c>
       <c r="P2" t="n">
-        <v>193595</v>
+        <v>179826</v>
       </c>
       <c r="Q2" t="n">
-        <v>0.9999920129776001</v>
+        <v>0.999991774559021</v>
       </c>
       <c r="R2" t="n">
-        <v>0.9985478520393372</v>
+        <v>0.9560158252716064</v>
       </c>
       <c r="S2" t="n">
-        <v>0.9894867539405823</v>
+        <v>0.9047700166702271</v>
       </c>
       <c r="T2" t="n">
-        <v>0.9870399832725525</v>
+        <v>0.8545472025871277</v>
       </c>
       <c r="U2" t="n">
-        <v>0.997006893157959</v>
+        <v>0.690119206905365</v>
       </c>
       <c r="V2" t="n">
-        <v>0.9979951977729797</v>
+        <v>0.9011067152023315</v>
       </c>
       <c r="W2" t="n">
-        <v>0.9983858466148376</v>
+        <v>0.9311330318450928</v>
       </c>
       <c r="X2" t="n">
-        <v>6396483</v>
+        <v>6196071</v>
       </c>
       <c r="Y2" t="n">
         <v>0</v>
@@ -742,132 +742,132 @@
         <v>0</v>
       </c>
       <c r="AE2" t="n">
-        <v>6396483</v>
+        <v>6196071</v>
       </c>
       <c r="AF2" t="n">
-        <v>4818683</v>
+        <v>4703530</v>
       </c>
       <c r="AG2" t="n">
-        <v>3064228</v>
+        <v>2913724</v>
       </c>
       <c r="AH2" t="n">
-        <v>810684</v>
+        <v>795355</v>
       </c>
       <c r="AI2" t="n">
-        <v>59622</v>
+        <v>58547</v>
       </c>
       <c r="AJ2" t="n">
-        <v>462194</v>
+        <v>458410</v>
       </c>
       <c r="AK2" t="n">
-        <v>180610</v>
+        <v>180009</v>
       </c>
       <c r="AL2" t="n">
         <v>1</v>
       </c>
       <c r="AM2" t="n">
-        <v>0.9546757936477661</v>
+        <v>0.9562803506851196</v>
       </c>
       <c r="AN2" t="n">
-        <v>0.9121971130371094</v>
+        <v>0.9113104939460754</v>
       </c>
       <c r="AO2" t="n">
-        <v>0.8573558926582336</v>
+        <v>0.8592069745063782</v>
       </c>
       <c r="AP2" t="n">
-        <v>0.6597105264663696</v>
+        <v>0.6631290316581726</v>
       </c>
       <c r="AQ2" t="n">
-        <v>0.9016343355178833</v>
+        <v>0.9023215174674988</v>
       </c>
       <c r="AR2" t="n">
-        <v>0.9313058257102966</v>
+        <v>0.931419849395752</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="n">
-        <v>0.0001053473441459384</v>
+        <v>0.002005508106422849</v>
       </c>
       <c r="B3" t="n">
-        <v>0.002041279598486683</v>
+        <v>0.00203137334927394</v>
       </c>
       <c r="C3" t="n">
         <v>0</v>
       </c>
       <c r="D3" t="n">
-        <v>5013592</v>
+        <v>4690075</v>
       </c>
       <c r="E3" t="n">
-        <v>21101</v>
+        <v>209541</v>
       </c>
       <c r="F3" t="n">
-        <v>4</v>
+        <v>8428</v>
       </c>
       <c r="G3" t="n">
-        <v>0</v>
+        <v>3627</v>
       </c>
       <c r="H3" t="n">
-        <v>0</v>
+        <v>84</v>
       </c>
       <c r="I3" t="n">
-        <v>0</v>
+        <v>22</v>
       </c>
       <c r="J3" t="n">
-        <v>10149066</v>
+        <v>9831078</v>
       </c>
       <c r="K3" t="n">
-        <v>11503612</v>
+        <v>10899643</v>
       </c>
       <c r="L3" t="n">
-        <v>13140373</v>
+        <v>12517633</v>
       </c>
       <c r="M3" t="n">
-        <v>15586139</v>
+        <v>14966018</v>
       </c>
       <c r="N3" t="n">
-        <v>16454882</v>
+        <v>15915395</v>
       </c>
       <c r="O3" t="n">
-        <v>16031399</v>
+        <v>15468531</v>
       </c>
       <c r="P3" t="n">
-        <v>16351237</v>
+        <v>15820637</v>
       </c>
       <c r="Q3" t="n">
         <v>1</v>
       </c>
       <c r="R3" t="n">
-        <v>0.9958080649375916</v>
+        <v>0.9548631906509399</v>
       </c>
       <c r="S3" t="n">
-        <v>0.9977985024452209</v>
+        <v>0.9107649922370911</v>
       </c>
       <c r="T3" t="n">
-        <v>0.9852872490882874</v>
+        <v>0.8521082997322083</v>
       </c>
       <c r="U3" t="n">
-        <v>0.8503541946411133</v>
+        <v>0.5900528430938721</v>
       </c>
       <c r="V3" t="n">
-        <v>0.999148428440094</v>
+        <v>0.9015480875968933</v>
       </c>
       <c r="W3" t="n">
-        <v>0.9976552724838257</v>
+        <v>0.9304729700088501</v>
       </c>
       <c r="X3" t="n">
         <v>0</v>
       </c>
       <c r="Y3" t="n">
-        <v>4818683</v>
+        <v>4703530</v>
       </c>
       <c r="Z3" t="n">
-        <v>200386</v>
+        <v>193315</v>
       </c>
       <c r="AA3" t="n">
-        <v>8658</v>
+        <v>8236</v>
       </c>
       <c r="AB3" t="n">
-        <v>6929</v>
+        <v>6655</v>
       </c>
       <c r="AC3" t="n">
         <v>11</v>
@@ -876,335 +876,335 @@
         <v>30</v>
       </c>
       <c r="AE3" t="n">
-        <v>10149117</v>
+        <v>9831129</v>
       </c>
       <c r="AF3" t="n">
-        <v>11282131</v>
+        <v>10900385</v>
       </c>
       <c r="AG3" t="n">
-        <v>12881150</v>
+        <v>12541068</v>
       </c>
       <c r="AH3" t="n">
-        <v>15463514</v>
+        <v>14970104</v>
       </c>
       <c r="AI3" t="n">
-        <v>16424359</v>
+        <v>15909071</v>
       </c>
       <c r="AJ3" t="n">
-        <v>15982005</v>
+        <v>15469206</v>
       </c>
       <c r="AK3" t="n">
-        <v>16338228</v>
+        <v>15820683</v>
       </c>
       <c r="AL3" t="n">
         <v>1</v>
       </c>
       <c r="AM3" t="n">
-        <v>0.9570949077606201</v>
+        <v>0.9576025009155273</v>
       </c>
       <c r="AN3" t="n">
-        <v>0.9094000458717346</v>
+        <v>0.9098091721534729</v>
       </c>
       <c r="AO3" t="n">
-        <v>0.8558678030967712</v>
+        <v>0.8582047820091248</v>
       </c>
       <c r="AP3" t="n">
-        <v>0.6589012742042542</v>
+        <v>0.6623938083648682</v>
       </c>
       <c r="AQ3" t="n">
-        <v>0.9006627202033997</v>
+        <v>0.9017251133918762</v>
       </c>
       <c r="AR3" t="n">
-        <v>0.9307395219802856</v>
+        <v>0.931419849395752</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="n">
-        <v>0.005149710689416298</v>
+        <v>0.03239797707621819</v>
       </c>
       <c r="B4" t="n">
-        <v>0.032156447865956</v>
+        <v>0.03199827809878473</v>
       </c>
       <c r="C4" t="n">
         <v>0</v>
       </c>
       <c r="D4" t="n">
-        <v>7237</v>
+        <v>201911</v>
       </c>
       <c r="E4" t="n">
-        <v>3362087</v>
+        <v>2916785</v>
       </c>
       <c r="F4" t="n">
-        <v>181</v>
+        <v>79974</v>
       </c>
       <c r="G4" t="n">
-        <v>0</v>
+        <v>2696</v>
       </c>
       <c r="H4" t="n">
-        <v>0</v>
+        <v>1138</v>
       </c>
       <c r="I4" t="n">
-        <v>0</v>
+        <v>62</v>
       </c>
       <c r="J4" t="n">
         <v>51</v>
       </c>
       <c r="K4" t="n">
-        <v>7291</v>
+        <v>215780</v>
       </c>
       <c r="L4" t="n">
-        <v>35722</v>
+        <v>307001</v>
       </c>
       <c r="M4" t="n">
-        <v>12254</v>
+        <v>134416</v>
       </c>
       <c r="N4" t="n">
-        <v>231</v>
+        <v>23418</v>
       </c>
       <c r="O4" t="n">
-        <v>1030</v>
+        <v>50299</v>
       </c>
       <c r="P4" t="n">
-        <v>313</v>
+        <v>13300</v>
       </c>
       <c r="Q4" t="n">
-        <v>0.9999960064888</v>
+        <v>0.9999958872795105</v>
       </c>
       <c r="R4" t="n">
-        <v>0.9971760511398315</v>
+        <v>0.9554391503334045</v>
       </c>
       <c r="S4" t="n">
-        <v>0.9936252236366272</v>
+        <v>0.907757580280304</v>
       </c>
       <c r="T4" t="n">
-        <v>0.9861628413200378</v>
+        <v>0.8533260226249695</v>
       </c>
       <c r="U4" t="n">
-        <v>0.9178595542907715</v>
+        <v>0.6361750960350037</v>
       </c>
       <c r="V4" t="n">
-        <v>0.998571515083313</v>
+        <v>0.90132737159729</v>
       </c>
       <c r="W4" t="n">
-        <v>0.9980204105377197</v>
+        <v>0.9308028817176819</v>
       </c>
       <c r="X4" t="n">
         <v>0</v>
       </c>
       <c r="Y4" t="n">
-        <v>213818</v>
+        <v>200856</v>
       </c>
       <c r="Z4" t="n">
-        <v>3064228</v>
+        <v>2913724</v>
       </c>
       <c r="AA4" t="n">
-        <v>84403</v>
+        <v>81391</v>
       </c>
       <c r="AB4" t="n">
-        <v>5710</v>
+        <v>5409</v>
       </c>
       <c r="AC4" t="n">
-        <v>1273</v>
+        <v>1118</v>
       </c>
       <c r="AD4" t="n">
-        <v>73</v>
+        <v>68</v>
       </c>
       <c r="AE4" t="n">
         <v>0</v>
       </c>
       <c r="AF4" t="n">
-        <v>228772</v>
+        <v>215038</v>
       </c>
       <c r="AG4" t="n">
-        <v>294945</v>
+        <v>283566</v>
       </c>
       <c r="AH4" t="n">
-        <v>134879</v>
+        <v>130330</v>
       </c>
       <c r="AI4" t="n">
-        <v>30754</v>
+        <v>29742</v>
       </c>
       <c r="AJ4" t="n">
-        <v>50424</v>
+        <v>49624</v>
       </c>
       <c r="AK4" t="n">
-        <v>13322</v>
+        <v>13254</v>
       </c>
       <c r="AL4" t="n">
         <v>1</v>
       </c>
       <c r="AM4" t="n">
-        <v>0.9558838605880737</v>
+        <v>0.9569409489631653</v>
       </c>
       <c r="AN4" t="n">
-        <v>0.9107964634895325</v>
+        <v>0.9105592370033264</v>
       </c>
       <c r="AO4" t="n">
-        <v>0.8566111922264099</v>
+        <v>0.8587056398391724</v>
       </c>
       <c r="AP4" t="n">
-        <v>0.6593056321144104</v>
+        <v>0.6627611517906189</v>
       </c>
       <c r="AQ4" t="n">
-        <v>0.90114825963974</v>
+        <v>0.9020231962203979</v>
       </c>
       <c r="AR4" t="n">
-        <v>0.931022584438324</v>
+        <v>0.931419849395752</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr"/>
       <c r="B5" t="inlineStr"/>
       <c r="C5" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D5" t="n">
-        <v>40</v>
+        <v>7728</v>
       </c>
       <c r="E5" t="n">
-        <v>13827</v>
+        <v>90351</v>
       </c>
       <c r="F5" t="n">
-        <v>933271</v>
+        <v>789705</v>
       </c>
       <c r="G5" t="n">
-        <v>69</v>
+        <v>9301</v>
       </c>
       <c r="H5" t="n">
-        <v>0</v>
+        <v>29050</v>
       </c>
       <c r="I5" t="n">
-        <v>0</v>
+        <v>630</v>
       </c>
       <c r="J5" t="n">
         <v>0</v>
       </c>
       <c r="K5" t="n">
-        <v>21105</v>
+        <v>221702</v>
       </c>
       <c r="L5" t="n">
-        <v>7418</v>
+        <v>285781</v>
       </c>
       <c r="M5" t="n">
-        <v>13936</v>
+        <v>137061</v>
       </c>
       <c r="N5" t="n">
-        <v>13541</v>
+        <v>36234</v>
       </c>
       <c r="O5" t="n">
-        <v>437</v>
+        <v>50050</v>
       </c>
       <c r="P5" t="n">
-        <v>455</v>
+        <v>13437</v>
       </c>
       <c r="Q5" t="n">
-        <v>0.9999969005584717</v>
+        <v>0.9999968409538269</v>
       </c>
       <c r="R5" t="n">
-        <v>0.9982837438583374</v>
+        <v>0.972703754901886</v>
       </c>
       <c r="S5" t="n">
-        <v>0.9973926544189453</v>
+        <v>0.9630140066146851</v>
       </c>
       <c r="T5" t="n">
-        <v>0.9984170794487</v>
+        <v>0.9830614924430847</v>
       </c>
       <c r="U5" t="n">
-        <v>0.9991676211357117</v>
+        <v>0.9962780475616455</v>
       </c>
       <c r="V5" t="n">
-        <v>0.9999113082885742</v>
+        <v>0.9937388300895691</v>
       </c>
       <c r="W5" t="n">
-        <v>0.99995356798172</v>
+        <v>0.9983317852020264</v>
       </c>
       <c r="X5" t="n">
         <v>0</v>
       </c>
       <c r="Y5" t="n">
-        <v>8236</v>
+        <v>7796</v>
       </c>
       <c r="Z5" t="n">
-        <v>88208</v>
+        <v>84121</v>
       </c>
       <c r="AA5" t="n">
-        <v>810684</v>
+        <v>795355</v>
       </c>
       <c r="AB5" t="n">
-        <v>10081</v>
+        <v>9865</v>
       </c>
       <c r="AC5" t="n">
-        <v>29357</v>
+        <v>28996</v>
       </c>
       <c r="AD5" t="n">
-        <v>641</v>
+        <v>633</v>
       </c>
       <c r="AE5" t="n">
         <v>0</v>
       </c>
       <c r="AF5" t="n">
-        <v>216014</v>
+        <v>208247</v>
       </c>
       <c r="AG5" t="n">
-        <v>305277</v>
+        <v>288842</v>
       </c>
       <c r="AH5" t="n">
-        <v>136523</v>
+        <v>131411</v>
       </c>
       <c r="AI5" t="n">
-        <v>30865</v>
+        <v>29840</v>
       </c>
       <c r="AJ5" t="n">
-        <v>50977</v>
+        <v>49960</v>
       </c>
       <c r="AK5" t="n">
-        <v>13440</v>
+        <v>13254</v>
       </c>
       <c r="AL5" t="n">
         <v>1</v>
       </c>
       <c r="AM5" t="n">
-        <v>0.9731175899505615</v>
+        <v>0.9735895991325378</v>
       </c>
       <c r="AN5" t="n">
-        <v>0.9637231826782227</v>
+        <v>0.9642851948738098</v>
       </c>
       <c r="AO5" t="n">
-        <v>0.9835967421531677</v>
+        <v>0.9836689233779907</v>
       </c>
       <c r="AP5" t="n">
-        <v>0.996275782585144</v>
+        <v>0.9962824583053589</v>
       </c>
       <c r="AQ5" t="n">
-        <v>0.9938714504241943</v>
+        <v>0.9937865734100342</v>
       </c>
       <c r="AR5" t="n">
-        <v>0.9983825087547302</v>
+        <v>0.9983460903167725</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr"/>
       <c r="B6" t="inlineStr"/>
       <c r="C6" t="n">
-        <v>10</v>
+        <v>20</v>
       </c>
       <c r="D6" t="n">
-        <v>14</v>
+        <v>6121</v>
       </c>
       <c r="E6" t="n">
-        <v>794</v>
+        <v>6196</v>
       </c>
       <c r="F6" t="n">
-        <v>12066</v>
+        <v>16118</v>
       </c>
       <c r="G6" t="n">
-        <v>76946</v>
+        <v>52153</v>
       </c>
       <c r="H6" t="n">
-        <v>623</v>
+        <v>7303</v>
       </c>
       <c r="I6" t="n">
-        <v>34</v>
+        <v>476</v>
       </c>
       <c r="J6" t="inlineStr"/>
       <c r="K6" t="inlineStr"/>
@@ -1224,22 +1224,22 @@
         <v>0</v>
       </c>
       <c r="Y6" t="n">
-        <v>6682</v>
+        <v>6351</v>
       </c>
       <c r="Z6" t="n">
-        <v>5459</v>
+        <v>5240</v>
       </c>
       <c r="AA6" t="n">
-        <v>11184</v>
+        <v>10819</v>
       </c>
       <c r="AB6" t="n">
-        <v>59622</v>
+        <v>58547</v>
       </c>
       <c r="AC6" t="n">
-        <v>7054</v>
+        <v>6949</v>
       </c>
       <c r="AD6" t="n">
-        <v>486</v>
+        <v>481</v>
       </c>
       <c r="AE6" t="inlineStr"/>
       <c r="AF6" t="inlineStr"/>
@@ -1260,25 +1260,25 @@
       <c r="A7" t="inlineStr"/>
       <c r="B7" t="inlineStr"/>
       <c r="C7" t="n">
-        <v>5</v>
+        <v>9</v>
       </c>
       <c r="D7" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="E7" t="n">
-        <v>0</v>
+        <v>814</v>
       </c>
       <c r="F7" t="n">
-        <v>0</v>
+        <v>29565</v>
       </c>
       <c r="G7" t="n">
-        <v>153</v>
+        <v>7549</v>
       </c>
       <c r="H7" t="n">
-        <v>512734</v>
+        <v>458320</v>
       </c>
       <c r="I7" t="n">
-        <v>279</v>
+        <v>12110</v>
       </c>
       <c r="J7" t="inlineStr"/>
       <c r="K7" t="inlineStr"/>
@@ -1298,22 +1298,22 @@
         <v>0</v>
       </c>
       <c r="Y7" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="Z7" t="n">
-        <v>810</v>
+        <v>809</v>
       </c>
       <c r="AA7" t="n">
-        <v>30300</v>
+        <v>29554</v>
       </c>
       <c r="AB7" t="n">
-        <v>7767</v>
+        <v>7548</v>
       </c>
       <c r="AC7" t="n">
-        <v>462194</v>
+        <v>458410</v>
       </c>
       <c r="AD7" t="n">
-        <v>12092</v>
+        <v>12042</v>
       </c>
       <c r="AE7" t="inlineStr"/>
       <c r="AF7" t="inlineStr"/>
@@ -1334,25 +1334,25 @@
       <c r="A8" t="inlineStr"/>
       <c r="B8" t="inlineStr"/>
       <c r="C8" t="n">
-        <v>36</v>
+        <v>21</v>
       </c>
       <c r="D8" t="n">
-        <v>0</v>
+        <v>17</v>
       </c>
       <c r="E8" t="n">
-        <v>0</v>
+        <v>99</v>
       </c>
       <c r="F8" t="n">
-        <v>3</v>
+        <v>331</v>
       </c>
       <c r="G8" t="n">
-        <v>9</v>
+        <v>245</v>
       </c>
       <c r="H8" t="n">
-        <v>407</v>
+        <v>12724</v>
       </c>
       <c r="I8" t="n">
-        <v>193595</v>
+        <v>179826</v>
       </c>
       <c r="J8" t="inlineStr"/>
       <c r="K8" t="inlineStr"/>
@@ -1375,19 +1375,19 @@
         <v>28</v>
       </c>
       <c r="Z8" t="n">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="AA8" t="n">
-        <v>334</v>
+        <v>330</v>
       </c>
       <c r="AB8" t="n">
-        <v>267</v>
+        <v>265</v>
       </c>
       <c r="AC8" t="n">
-        <v>12729</v>
+        <v>12550</v>
       </c>
       <c r="AD8" t="n">
-        <v>180610</v>
+        <v>180009</v>
       </c>
       <c r="AE8" t="inlineStr"/>
       <c r="AF8" t="inlineStr"/>

</xml_diff>